<commit_message>
generacion de confmato de constatacion
</commit_message>
<xml_diff>
--- a/PLANTILLA_FC.xlsx
+++ b/PLANTILLA_FC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e1ed37ae7f44536/Documentos/CONSTATACION/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{7CA578D7-45B3-4342-A4B9-AF13468BBEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F89113EB-2917-43D2-B82D-DFBA9A387002}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{7CA578D7-45B3-4342-A4B9-AF13468BBEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0E5E4C5-069D-4788-9AE9-7832EB40C929}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{945A3697-4670-429F-BBCC-7606A0933988}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{945A3697-4670-429F-BBCC-7606A0933988}"/>
   </bookViews>
   <sheets>
     <sheet name="ID EMPRESA" sheetId="2" r:id="rId1"/>
@@ -78,12 +78,10 @@
     <t>PARTIDA</t>
   </si>
   <si>
-    <t>SIN 
-AGUA</t>
-  </si>
-  <si>
-    <t>SIN 
-SANEAMIENTO</t>
+    <t>SIN AGUA</t>
+  </si>
+  <si>
+    <t>SIN SANEAMIENTO</t>
   </si>
   <si>
     <t>DISTRITO</t>
@@ -96,7 +94,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,8 +118,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,37 +166,40 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor theme="9"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="4" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -226,89 +265,384 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Cálculo" xfId="1" builtinId="22"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
+  <dxfs count="25">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
         </left>
         <right style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </right>
         <top style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </top>
         <bottom style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </bottom>
         <vertical style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </vertical>
         <horizontal style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </horizontal>
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color rgb="FF000000"/>
+        </vertical>
+        <horizontal style="thin">
+          <color rgb="FF000000"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -325,7 +659,16 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -342,6 +685,16 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment wrapText="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -358,7 +711,16 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -375,7 +737,16 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -392,6 +763,16 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment wrapText="1"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -436,10 +817,18 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <font>
+        <sz val="14"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+        <color theme="0"/>
+      </font>
+      <alignment horizontal="center"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -464,25 +853,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4ADF3151-3637-416B-BC56-8CBB1D14AC3E}" name="Tabla2" displayName="Tabla2" ref="A1:I2" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4ADF3151-3637-416B-BC56-8CBB1D14AC3E}" name="Tabla2" displayName="Tabla2" ref="A1:I2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" headerRowBorderDxfId="21" tableBorderDxfId="22" totalsRowBorderDxfId="20">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{446D464C-8835-4266-A9A2-58FA1FCCBDCB}" name="DNI" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{1E7A6524-D320-4D12-A5DA-B020D8CA46C3}" name="RL" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{DE0C6670-2DFB-4B60-AEFC-8A5BDFDA2E05}" name="ET" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{91847190-97A2-45DA-BEDB-6643175BF8B9}" name="DIR GERET" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{1337F15A-CB87-423E-87A6-F921AFD933BC}" name="RUC" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{4F1E1F9D-3EEE-47AB-84C6-595829B6E95D}" name="COD REG" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{B268CBFC-1E06-430D-91F4-DB5AB041D323}" name="DNI ING" dataDxfId="5" dataCellStyle="Cálculo"/>
-    <tableColumn id="9" xr3:uid="{31E360B3-0870-4FEF-AD27-1137A3B42C61}" name="CIP" dataDxfId="4" dataCellStyle="Cálculo"/>
-    <tableColumn id="10" xr3:uid="{822C8717-48E8-4439-A05E-B3AD29A6B828}" name="NOMBRE ING" dataDxfId="3" dataCellStyle="Cálculo"/>
+    <tableColumn id="1" xr3:uid="{446D464C-8835-4266-A9A2-58FA1FCCBDCB}" name="DNI" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{1E7A6524-D320-4D12-A5DA-B020D8CA46C3}" name="RL" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{DE0C6670-2DFB-4B60-AEFC-8A5BDFDA2E05}" name="ET" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{91847190-97A2-45DA-BEDB-6643175BF8B9}" name="DIR GERET" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{1337F15A-CB87-423E-87A6-F921AFD933BC}" name="RUC" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{4F1E1F9D-3EEE-47AB-84C6-595829B6E95D}" name="COD REG" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{B268CBFC-1E06-430D-91F4-DB5AB041D323}" name="DNI ING" dataDxfId="13" dataCellStyle="Cálculo"/>
+    <tableColumn id="9" xr3:uid="{31E360B3-0870-4FEF-AD27-1137A3B42C61}" name="CIP" dataDxfId="12" dataCellStyle="Cálculo"/>
+    <tableColumn id="10" xr3:uid="{822C8717-48E8-4439-A05E-B3AD29A6B828}" name="NOMBRE ING" dataDxfId="11" dataCellStyle="Cálculo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A74F8C3-E560-4B8A-A8B2-B1A5C3CB5C21}" name="Tabla1" displayName="Tabla1" ref="A1:G17" totalsRowShown="0">
-  <autoFilter ref="A1:G17" xr:uid="{9A74F8C3-E560-4B8A-A8B2-B1A5C3CB5C21}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A74F8C3-E560-4B8A-A8B2-B1A5C3CB5C21}" name="Tabla1" displayName="Tabla1" ref="A1:I21" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I21" xr:uid="{9A74F8C3-E560-4B8A-A8B2-B1A5C3CB5C21}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -490,17 +879,21 @@
     <filterColumn colId="4" hiddenButton="1"/>
     <filterColumn colId="5" hiddenButton="1"/>
     <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{875342A5-94C6-4EED-AC3D-C692FD466BB6}" name="ITEM"/>
-    <tableColumn id="2" xr3:uid="{562BE676-2409-4E77-BC7F-5972BEB37BC1}" name="DNI"/>
-    <tableColumn id="3" xr3:uid="{B800AA76-8009-4EA7-80A2-F2C439A59B8C}" name="GRUPO FAMILIAR"/>
-    <tableColumn id="4" xr3:uid="{939E6FDD-8378-4578-A6E1-C27052D54DD9}" name="DIRECCION PREDIO"/>
-    <tableColumn id="5" xr3:uid="{B0C21390-3D79-4460-A76F-533123278F33}" name="PARTIDA" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{F4801E72-7DE6-45D6-9D5C-5E9C6453A2B9}" name="SIN _x000a_AGUA" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{2D2BEEE8-EF72-4AB9-B0BE-E9A6589AEC1F}" name="SIN _x000a_SANEAMIENTO" dataDxfId="0"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{875342A5-94C6-4EED-AC3D-C692FD466BB6}" name="ITEM" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{562BE676-2409-4E77-BC7F-5972BEB37BC1}" name="DNI" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{B800AA76-8009-4EA7-80A2-F2C439A59B8C}" name="GRUPO FAMILIAR" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{939E6FDD-8378-4578-A6E1-C27052D54DD9}" name="DIRECCION PREDIO" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{B0C21390-3D79-4460-A76F-533123278F33}" name="PARTIDA" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{F4801E72-7DE6-45D6-9D5C-5E9C6453A2B9}" name="SIN AGUA" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{2D2BEEE8-EF72-4AB9-B0BE-E9A6589AEC1F}" name="SIN SANEAMIENTO" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{84DAC141-9FC7-45B2-B817-6064650DA21F}" name="DISTRITO" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{1856E2ED-A01E-4BD0-97F6-36AF90395882}" name="PROVINCIA" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -801,58 +1194,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74423D49-8C24-4D8D-8610-FB0C5D6518B1}">
-  <dimension ref="A1:I2"/>
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.85546875" customWidth="1"/>
     <col min="5" max="5" width="14.85546875" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="9" max="9" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:9" s="5" customFormat="1" ht="18.75">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-    </row>
+    <row r="2" spans="1:9" s="10" customFormat="1" ht="45" customHeight="1">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" ht="18.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -863,212 +1262,311 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{442AAB1F-60B3-4231-AC22-61841D5D6780}">
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="89.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" customWidth="1"/>
+    <col min="3" max="3" width="51" customWidth="1"/>
+    <col min="4" max="4" width="48.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" ht="30.75">
+      <c r="A1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="17" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2">
+      <c r="A2" s="14">
         <v>1</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3">
+      <c r="A3" s="14">
         <v>2</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4">
+      <c r="A4" s="14">
         <v>3</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5">
+      <c r="A5" s="14">
         <v>4</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6">
+      <c r="A6" s="14">
         <v>5</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7">
+      <c r="A7" s="14">
         <v>6</v>
       </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8">
+      <c r="A8" s="14">
         <v>7</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9">
+      <c r="A9" s="14">
         <v>8</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10">
+      <c r="A10" s="14">
         <v>9</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11">
+      <c r="A11" s="14">
         <v>10</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12">
+      <c r="A12" s="14">
         <v>11</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13">
+      <c r="A13" s="14">
         <v>12</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14">
+      <c r="A14" s="14">
         <v>13</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15">
+      <c r="A15" s="14">
         <v>14</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16">
+      <c r="A16" s="14">
         <v>15</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17">
+      <c r="A17" s="14">
         <v>16</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="14">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="14">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="C20" s="1"/>
+      <c r="A20" s="14">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
     </row>
     <row r="21" spans="1:9">
-      <c r="C21" s="1"/>
+      <c r="A21" s="14">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
     </row>
     <row r="23" spans="1:9">
       <c r="C23" s="1"/>

</xml_diff>